<commit_message>
data: daily one-to-two V1 scan and web result
</commit_message>
<xml_diff>
--- a/docs/downloads/latest.xlsx
+++ b/docs/downloads/latest.xlsx
@@ -93,7 +93,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L138"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
@@ -3559,13 +3559,3955 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B66" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C66" s="0">
+        <v>1</v>
+      </c>
+      <c r="D66" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">000607</t>
+        </is>
+      </c>
+      <c r="E66" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">华媒控股</t>
+        </is>
+      </c>
+      <c r="F66" s="0">
+        <v>4.53</v>
+      </c>
+      <c r="G66" s="4">
+        <v>0.09951456310679617</v>
+      </c>
+      <c r="H66" s="4">
+        <v>0.4652418066589123</v>
+      </c>
+      <c r="I66" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J66" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 华媒控股（000607）归入“文化传媒+AI应用+国企”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K66" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。今日开盘已接近涨停价，开盘强度较高（开盘涨幅 10.0%）。截至运行时成交量约为20日均量的 1.1 倍，量能未出现极端放大。短中期均线保持多头排列，价格结构与趋势方向一致。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L66" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B67" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C67" s="0">
+        <v>2</v>
+      </c>
+      <c r="D67" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600825</t>
+        </is>
+      </c>
+      <c r="E67" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">新华传媒</t>
+        </is>
+      </c>
+      <c r="F67" s="0">
+        <v>5.84</v>
+      </c>
+      <c r="G67" s="4">
+        <v>0.09981167608286266</v>
+      </c>
+      <c r="H67" s="4">
+        <v>0.46339117758857357</v>
+      </c>
+      <c r="I67" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 新华传媒（600825）归入“资产重组+复牌+图书发行+上海国资”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。今日开盘已接近涨停价，开盘强度较高（开盘涨幅 10.0%）。截至运行时成交量约为20日均量的 0.3 倍，量能未出现极端放大。短中期均线保持多头排列，价格结构与趋势方向一致。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L67" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C68" s="0">
+        <v>3</v>
+      </c>
+      <c r="D68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002614</t>
+        </is>
+      </c>
+      <c r="E68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">奥佳华</t>
+        </is>
+      </c>
+      <c r="F68" s="0">
+        <v>6.25</v>
+      </c>
+      <c r="G68" s="4">
+        <v>0.10035211267605648</v>
+      </c>
+      <c r="H68" s="4">
+        <v>0.37674420222437527</v>
+      </c>
+      <c r="I68" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 奥佳华（002614）归入“股份转让+具身智能+智能按摩椅+大健康品牌”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K68" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。今日开盘已接近涨停价，开盘强度较高（开盘涨幅 9.2%）。截至运行时成交量约为20日均量的 0.7 倍，量能未出现极端放大。5日均线仍高于10日均线，但中期趋势强度一般。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L68" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C69" s="0">
+        <v>4</v>
+      </c>
+      <c r="D69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600743</t>
+        </is>
+      </c>
+      <c r="E69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">华远控股</t>
+        </is>
+      </c>
+      <c r="F69" s="0">
+        <v>2.33</v>
+      </c>
+      <c r="G69" s="4">
+        <v>0.09905660377358494</v>
+      </c>
+      <c r="H69" s="4">
+        <v>0.33858885816024553</v>
+      </c>
+      <c r="I69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 华远控股（600743）归入“控股变更+物业管理+酒店管理”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K69" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。今日开盘已接近涨停价，开盘强度较高（开盘涨幅 9.9%）。截至运行时成交量约为20日均量的 0.5 倍，量能未出现极端放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L69" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C70" s="0">
+        <v>5</v>
+      </c>
+      <c r="D70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600301</t>
+        </is>
+      </c>
+      <c r="E70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">华锡有色</t>
+        </is>
+      </c>
+      <c r="F70" s="0">
+        <v>49.97</v>
+      </c>
+      <c r="G70" s="4">
+        <v>0.09993396434074399</v>
+      </c>
+      <c r="H70" s="4">
+        <v>0.2342618480988038</v>
+      </c>
+      <c r="I70" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 华锡有色（600301）归入“控制权变更+锡锑铟+业绩增长”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K70" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。今日开盘已接近涨停价，开盘强度较高（开盘涨幅 10.0%）。截至运行时成交量约为20日均量的 0.6 倍，量能未出现极端放大。5日均线仍高于10日均线，但中期趋势强度一般。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L70" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C71" s="0">
+        <v>6</v>
+      </c>
+      <c r="D71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002303</t>
+        </is>
+      </c>
+      <c r="E71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">美盈森</t>
+        </is>
+      </c>
+      <c r="F71" s="0">
+        <v>6.27</v>
+      </c>
+      <c r="G71" s="4">
+        <v>0.09999999999999985</v>
+      </c>
+      <c r="H71" s="4">
+        <v>0.1950828698236118</v>
+      </c>
+      <c r="I71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 美盈森（002303）归入“包装一体化+消费电子包装+模切业务+海外产能”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K71" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 0.6 倍，量能未出现极端放大。短中期均线保持多头排列，价格结构与趋势方向一致。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L71" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C72" s="0">
+        <v>7</v>
+      </c>
+      <c r="D72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002585</t>
+        </is>
+      </c>
+      <c r="E72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">双星新材</t>
+        </is>
+      </c>
+      <c r="F72" s="0">
+        <v>12.71</v>
+      </c>
+      <c r="G72" s="4">
+        <v>0.10043290043290053</v>
+      </c>
+      <c r="H72" s="4">
+        <v>0.18885269109174457</v>
+      </c>
+      <c r="I72" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J72" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 双星新材（002585）归入“MLCC离型膜+复合铜箔+聚酯薄膜”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K72" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.5 倍，存在明显放量。短中期均线保持多头排列，价格结构与趋势方向一致。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L72" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C73" s="0">
+        <v>8</v>
+      </c>
+      <c r="D73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002172</t>
+        </is>
+      </c>
+      <c r="E73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">澳洋健康</t>
+        </is>
+      </c>
+      <c r="F73" s="0">
+        <v>5.81</v>
+      </c>
+      <c r="G73" s="4">
+        <v>0.10037878787878786</v>
+      </c>
+      <c r="H73" s="4">
+        <v>0.17677673435453747</v>
+      </c>
+      <c r="I73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 澳洋健康（002172）归入“脑机接口+医疗服务+国资”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K73" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 0.6 倍，量能未出现极端放大。短中期均线保持多头排列，价格结构与趋势方向一致。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L73" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C74" s="0">
+        <v>9</v>
+      </c>
+      <c r="D74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">001201</t>
+        </is>
+      </c>
+      <c r="E74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">东瑞股份</t>
+        </is>
+      </c>
+      <c r="F74" s="0">
+        <v>16.08</v>
+      </c>
+      <c r="G74" s="4">
+        <v>0.09986320109439116</v>
+      </c>
+      <c r="H74" s="4">
+        <v>0.15556029997125023</v>
+      </c>
+      <c r="I74" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J74" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 东瑞股份（001201）归入“生猪养殖+供港活猪+降本增效”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K74" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 2.1 倍，资金参与度显著放大。短中期均线保持多头排列，价格结构与趋势方向一致。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L74" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C75" s="0">
+        <v>10</v>
+      </c>
+      <c r="D75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002084</t>
+        </is>
+      </c>
+      <c r="E75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">海鸥住工</t>
+        </is>
+      </c>
+      <c r="F75" s="0">
+        <v>6.12</v>
+      </c>
+      <c r="G75" s="4">
+        <v>0.10071942446043171</v>
+      </c>
+      <c r="H75" s="4">
+        <v>0.1543190939107268</v>
+      </c>
+      <c r="I75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 海鸥住工（002084）归入“控制权拟变更+装配式厨卫+越南制造”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K75" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 0.6 倍，量能未出现极端放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L75" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C76" s="0">
+        <v>11</v>
+      </c>
+      <c r="D76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603042</t>
+        </is>
+      </c>
+      <c r="E76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">华脉科技</t>
+        </is>
+      </c>
+      <c r="F76" s="0">
+        <v>19.03</v>
+      </c>
+      <c r="G76" s="4">
+        <v>0.10000000000000009</v>
+      </c>
+      <c r="H76" s="4">
+        <v>0.14686166753756646</v>
+      </c>
+      <c r="I76" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J76" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 华脉科技（603042）归入“光纤光缆+扭亏为盈+6G布局”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K76" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.6 倍，存在明显放量。短中期均线保持多头排列，价格结构与趋势方向一致。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L76" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B77" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C77" s="0">
+        <v>12</v>
+      </c>
+      <c r="D77" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603663</t>
+        </is>
+      </c>
+      <c r="E77" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">三祥新材</t>
+        </is>
+      </c>
+      <c r="F77" s="0">
+        <v>49.82</v>
+      </c>
+      <c r="G77" s="4">
+        <v>0.1000220799293443</v>
+      </c>
+      <c r="H77" s="4">
+        <v>0.14652972517382876</v>
+      </c>
+      <c r="I77" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 三祥新材（603663）归入“锆铪分离+半导体+海绵锆”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K77" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.0 倍，量能未出现极端放大。短中期均线保持多头排列，价格结构与趋势方向一致。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L77" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B78" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C78" s="0">
+        <v>13</v>
+      </c>
+      <c r="D78" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002388</t>
+        </is>
+      </c>
+      <c r="E78" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">新亚制程</t>
+        </is>
+      </c>
+      <c r="F78" s="0">
+        <v>7.95</v>
+      </c>
+      <c r="G78" s="4">
+        <v>0.09958506224066375</v>
+      </c>
+      <c r="H78" s="4">
+        <v>0.1410810028618283</v>
+      </c>
+      <c r="I78" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J78" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 新亚制程（002388）归入“AI服务器电源+胶粘剂+六氟磷酸锂”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K78" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.3 倍，存在明显放量。短中期均线保持多头排列，价格结构与趋势方向一致。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L78" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B79" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C79" s="0">
+        <v>14</v>
+      </c>
+      <c r="D79" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002724</t>
+        </is>
+      </c>
+      <c r="E79" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">海洋王</t>
+        </is>
+      </c>
+      <c r="F79" s="0">
+        <v>7.84</v>
+      </c>
+      <c r="G79" s="4">
+        <v>0.09957924263674611</v>
+      </c>
+      <c r="H79" s="4">
+        <v>0.14094176062559174</v>
+      </c>
+      <c r="I79" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J79" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 海洋王（002724）归入“AI照明+工业照明+应急救援”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K79" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.5 倍，存在明显放量。短中期均线保持多头排列，价格结构与趋势方向一致。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L79" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B80" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C80" s="0">
+        <v>15</v>
+      </c>
+      <c r="D80" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603819</t>
+        </is>
+      </c>
+      <c r="E80" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">神力股份</t>
+        </is>
+      </c>
+      <c r="F80" s="0">
+        <v>17.33</v>
+      </c>
+      <c r="G80" s="4">
+        <v>0.10031746031746014</v>
+      </c>
+      <c r="H80" s="4">
+        <v>0.1360845517633556</v>
+      </c>
+      <c r="I80" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J80" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 神力股份（603819）归入“电机铁芯+风电+电梯配件+半年报增长”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K80" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.2 倍，量能未出现极端放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L80" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B81" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C81" s="0">
+        <v>16</v>
+      </c>
+      <c r="D81" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603319</t>
+        </is>
+      </c>
+      <c r="E81" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">XD美湖股份</t>
+        </is>
+      </c>
+      <c r="F81" s="0">
+        <v>32.18</v>
+      </c>
+      <c r="G81" s="4">
+        <v>0.10017094017094008</v>
+      </c>
+      <c r="H81" s="4">
+        <v>0.1345846761414189</v>
+      </c>
+      <c r="I81" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J81" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 XD美湖股份（603319）归入“机器人执行器+服务器液冷+泵类龙头”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K81" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.8 倍，资金参与度显著放大。短中期均线保持多头排列，价格结构与趋势方向一致。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L81" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B82" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C82" s="0">
+        <v>17</v>
+      </c>
+      <c r="D82" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002080</t>
+        </is>
+      </c>
+      <c r="E82" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中材科技</t>
+        </is>
+      </c>
+      <c r="F82" s="0">
+        <v>66.24</v>
+      </c>
+      <c r="G82" s="4">
+        <v>0.09996678844237783</v>
+      </c>
+      <c r="H82" s="4">
+        <v>0.1343407096372262</v>
+      </c>
+      <c r="I82" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J82" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 中材科技（002080）归入“低介电纤维布+高频高速PCB+玻纤主业”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K82" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 2.4 倍，资金参与度显著放大。短中期均线保持多头排列，价格结构与趋势方向一致。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L82" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B83" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C83" s="0">
+        <v>18</v>
+      </c>
+      <c r="D83" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002367</t>
+        </is>
+      </c>
+      <c r="E83" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">康力电梯</t>
+        </is>
+      </c>
+      <c r="F83" s="0">
+        <v>6.28</v>
+      </c>
+      <c r="G83" s="4">
+        <v>0.09982486865148864</v>
+      </c>
+      <c r="H83" s="4">
+        <v>0.13114815737366875</v>
+      </c>
+      <c r="I83" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J83" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 康力电梯（002367）归入“旧梯更新+轨道交通+智能电梯”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K83" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.9 倍，资金参与度显著放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L83" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B84" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C84" s="0">
+        <v>19</v>
+      </c>
+      <c r="D84" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">000560</t>
+        </is>
+      </c>
+      <c r="E84" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">我爱我家</t>
+        </is>
+      </c>
+      <c r="F84" s="0">
+        <v>3.19</v>
+      </c>
+      <c r="G84" s="4">
+        <v>0.10000000000000009</v>
+      </c>
+      <c r="H84" s="4">
+        <v>0.12987375444567673</v>
+      </c>
+      <c r="I84" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J84" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 我爱我家（000560）归入“房产经纪+AI应用+净利增长”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K84" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.0 倍，量能未出现极端放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L84" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日振幅较大</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B85" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C85" s="0">
+        <v>20</v>
+      </c>
+      <c r="D85" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600712</t>
+        </is>
+      </c>
+      <c r="E85" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">南宁百货</t>
+        </is>
+      </c>
+      <c r="F85" s="0">
+        <v>5.89</v>
+      </c>
+      <c r="G85" s="4">
+        <v>0.10093457943925245</v>
+      </c>
+      <c r="H85" s="4">
+        <v>0.12873773638560287</v>
+      </c>
+      <c r="I85" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 南宁百货（600712）归入“百货零售+平陆运河+扭亏为盈”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.8 倍，存在明显放量。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B86" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C86" s="0">
+        <v>21</v>
+      </c>
+      <c r="D86" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600664</t>
+        </is>
+      </c>
+      <c r="E86" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">哈药股份</t>
+        </is>
+      </c>
+      <c r="F86" s="0">
+        <v>8.25</v>
+      </c>
+      <c r="G86" s="4">
+        <v>0.10000000000000009</v>
+      </c>
+      <c r="H86" s="4">
+        <v>0.12766536973531</v>
+      </c>
+      <c r="I86" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J86" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 哈药股份（600664）归入“创新药研发+医药工业+业绩增长”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K86" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 0.5 倍，量能未出现极端放大。5日均线仍高于10日均线，但中期趋势强度一般。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L86" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B87" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C87" s="0">
+        <v>22</v>
+      </c>
+      <c r="D87" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">001234</t>
+        </is>
+      </c>
+      <c r="E87" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">泰慕士</t>
+        </is>
+      </c>
+      <c r="F87" s="0">
+        <v>26.59</v>
+      </c>
+      <c r="G87" s="4">
+        <v>0.10012412081092247</v>
+      </c>
+      <c r="H87" s="4">
+        <v>0.12764818270936235</v>
+      </c>
+      <c r="I87" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J87" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 泰慕士（001234）归入“针织服装+服装贴牌+广州国资入主”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K87" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 2.2 倍，资金参与度显著放大。短中期均线保持多头排列，价格结构与趋势方向一致。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L87" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B88" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C88" s="0">
+        <v>23</v>
+      </c>
+      <c r="D88" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002792</t>
+        </is>
+      </c>
+      <c r="E88" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通宇通讯</t>
+        </is>
+      </c>
+      <c r="F88" s="0">
+        <v>34.54</v>
+      </c>
+      <c r="G88" s="4">
+        <v>0.10000000000000009</v>
+      </c>
+      <c r="H88" s="4">
+        <v>0.12699105645561096</v>
+      </c>
+      <c r="I88" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J88" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 通宇通讯（002792）归入“卫星通信+基站天线+海外业务”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K88" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 2.6 倍，资金参与度显著放大。短中期均线保持多头排列，价格结构与趋势方向一致。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L88" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B89" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C89" s="0">
+        <v>24</v>
+      </c>
+      <c r="D89" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">001389</t>
+        </is>
+      </c>
+      <c r="E89" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">广合科技</t>
+        </is>
+      </c>
+      <c r="F89" s="0">
+        <v>185.93</v>
+      </c>
+      <c r="G89" s="4">
+        <v>0.09998225167130093</v>
+      </c>
+      <c r="H89" s="4">
+        <v>0.12614165188586235</v>
+      </c>
+      <c r="I89" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 广合科技（001389）归入“算力PCB+高端产能+业绩增长”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K89" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 2.1 倍，资金参与度显著放大。短中期均线保持多头排列，价格结构与趋势方向一致。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L89" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B90" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C90" s="0">
+        <v>25</v>
+      </c>
+      <c r="D90" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002963</t>
+        </is>
+      </c>
+      <c r="E90" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">豪尔赛</t>
+        </is>
+      </c>
+      <c r="F90" s="0">
+        <v>22.62</v>
+      </c>
+      <c r="G90" s="4">
+        <v>0.10019455252918297</v>
+      </c>
+      <c r="H90" s="4">
+        <v>0.1242262874871728</v>
+      </c>
+      <c r="I90" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J90" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 豪尔赛（002963）归入“智慧能源+照明工程+拟收购新能动力+澄清液冷”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K90" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 0.8 倍，量能未出现极端放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L90" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B91" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C91" s="0">
+        <v>26</v>
+      </c>
+      <c r="D91" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600857</t>
+        </is>
+      </c>
+      <c r="E91" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">宁波中百</t>
+        </is>
+      </c>
+      <c r="F91" s="0">
+        <v>23.41</v>
+      </c>
+      <c r="G91" s="4">
+        <v>0.10009398496240607</v>
+      </c>
+      <c r="H91" s="4">
+        <v>0.12335097963154369</v>
+      </c>
+      <c r="I91" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J91" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 宁波中百（600857）归入“商业零售+黄金珠宝+杭州金帝入主”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K91" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.0 倍，量能未出现极端放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L91" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B92" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C92" s="0">
+        <v>27</v>
+      </c>
+      <c r="D92" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002246</t>
+        </is>
+      </c>
+      <c r="E92" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">北化股份</t>
+        </is>
+      </c>
+      <c r="F92" s="0">
+        <v>26.27</v>
+      </c>
+      <c r="G92" s="4">
+        <v>0.10008375209380226</v>
+      </c>
+      <c r="H92" s="4">
+        <v>0.12259349734404079</v>
+      </c>
+      <c r="I92" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J92" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 北化股份（002246）归入“硝化棉+商业航天+央企”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K92" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 2.4 倍，资金参与度显著放大。短中期均线保持多头排列，价格结构与趋势方向一致。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L92" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B93" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C93" s="0">
+        <v>28</v>
+      </c>
+      <c r="D93" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603020</t>
+        </is>
+      </c>
+      <c r="E93" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">爱普股份</t>
+        </is>
+      </c>
+      <c r="F93" s="0">
+        <v>12.57</v>
+      </c>
+      <c r="G93" s="4">
+        <v>0.09973753280839892</v>
+      </c>
+      <c r="H93" s="4">
+        <v>0.12196322877452691</v>
+      </c>
+      <c r="I93" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J93" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 爱普股份（603020）归入“半导体材料+香精香料+鱼油原料”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K93" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 2.1 倍，资金参与度显著放大。短中期均线保持多头排列，价格结构与趋势方向一致。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L93" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B94" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C94" s="0">
+        <v>29</v>
+      </c>
+      <c r="D94" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">605566</t>
+        </is>
+      </c>
+      <c r="E94" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">福莱蒽特</t>
+        </is>
+      </c>
+      <c r="F94" s="0">
+        <v>30.44</v>
+      </c>
+      <c r="G94" s="4">
+        <v>0.10010842067220803</v>
+      </c>
+      <c r="H94" s="4">
+        <v>0.1216132115219928</v>
+      </c>
+      <c r="I94" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J94" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 福莱蒽特（605566）归入“分散染料+服务器采购+机器人皮肤”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K94" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.4 倍，存在明显放量。5日均线仍高于10日均线，但中期趋势强度一般。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L94" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B95" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C95" s="0">
+        <v>30</v>
+      </c>
+      <c r="D95" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">000020</t>
+        </is>
+      </c>
+      <c r="E95" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">深华发Ａ</t>
+        </is>
+      </c>
+      <c r="F95" s="0">
+        <v>14.26</v>
+      </c>
+      <c r="G95" s="4">
+        <v>0.10030864197530853</v>
+      </c>
+      <c r="H95" s="4">
+        <v>0.12084880643633285</v>
+      </c>
+      <c r="I95" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J95" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 深华发Ａ（000020）归入“定制显示器+深圳旧改+物业经营+注塑业务”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K95" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.1 倍，量能未出现极端放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L95" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B96" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C96" s="0">
+        <v>31</v>
+      </c>
+      <c r="D96" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600593</t>
+        </is>
+      </c>
+      <c r="E96" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">大连圣亚</t>
+        </is>
+      </c>
+      <c r="F96" s="0">
+        <v>48.57</v>
+      </c>
+      <c r="G96" s="4">
+        <v>0.10011325028312568</v>
+      </c>
+      <c r="H96" s="4">
+        <v>0.12028803328689865</v>
+      </c>
+      <c r="I96" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J96" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 大连圣亚（600593）归入“旅游经营+海洋公园+业绩扭亏”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K96" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 2.4 倍，资金参与度显著放大。5日均线仍高于10日均线，但中期趋势强度一般。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L96" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B97" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C97" s="0">
+        <v>32</v>
+      </c>
+      <c r="D97" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603151</t>
+        </is>
+      </c>
+      <c r="E97" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">邦基科技股份</t>
+        </is>
+      </c>
+      <c r="F97" s="0">
+        <v>18.35</v>
+      </c>
+      <c r="G97" s="4">
+        <v>0.10011990407673865</v>
+      </c>
+      <c r="H97" s="4">
+        <v>0.12016408243019151</v>
+      </c>
+      <c r="I97" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J97" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 邦基科技股份（603151）归入“猪饲料+生猪养殖+产业链一体化”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K97" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 0.8 倍，量能未出现极端放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L97" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B98" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C98" s="0">
+        <v>33</v>
+      </c>
+      <c r="D98" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002321</t>
+        </is>
+      </c>
+      <c r="E98" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">华英农业</t>
+        </is>
+      </c>
+      <c r="F98" s="0">
+        <v>2.3</v>
+      </c>
+      <c r="G98" s="4">
+        <v>0.10047846889952151</v>
+      </c>
+      <c r="H98" s="4">
+        <v>0.11799329681958166</v>
+      </c>
+      <c r="I98" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J98" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 华英农业（002321）归入“鸭业全产业链+羽绒出口+控制权变更”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K98" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 2.5 倍，资金参与度显著放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L98" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分；当日振幅较大</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B99" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C99" s="0">
+        <v>34</v>
+      </c>
+      <c r="D99" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603093</t>
+        </is>
+      </c>
+      <c r="E99" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">南华期货</t>
+        </is>
+      </c>
+      <c r="F99" s="0">
+        <v>13.99</v>
+      </c>
+      <c r="G99" s="4">
+        <v>0.09984276729559749</v>
+      </c>
+      <c r="H99" s="4">
+        <v>0.1178917621278945</v>
+      </c>
+      <c r="I99" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J99" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 南华期货（603093）归入“境外金融服务+境外清算+期货经纪”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K99" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.0 倍，量能未出现极端放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L99" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B100" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C100" s="0">
+        <v>35</v>
+      </c>
+      <c r="D100" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600721</t>
+        </is>
+      </c>
+      <c r="E100" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">百花医药</t>
+        </is>
+      </c>
+      <c r="F100" s="0">
+        <v>13.15</v>
+      </c>
+      <c r="G100" s="4">
+        <v>0.10041841004184103</v>
+      </c>
+      <c r="H100" s="4">
+        <v>0.11730331242139477</v>
+      </c>
+      <c r="I100" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J100" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 百花医药（600721）归入“CRO+复杂制剂+国资背景”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K100" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.0 倍，量能未出现极端放大。5日均线仍高于10日均线，但中期趋势强度一般。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L100" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B101" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C101" s="0">
+        <v>36</v>
+      </c>
+      <c r="D101" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603175</t>
+        </is>
+      </c>
+      <c r="E101" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">超颖电子</t>
+        </is>
+      </c>
+      <c r="F101" s="0">
+        <v>110.17</v>
+      </c>
+      <c r="G101" s="4">
+        <v>0.10004992511233146</v>
+      </c>
+      <c r="H101" s="4">
+        <v>0.11683520091249867</v>
+      </c>
+      <c r="I101" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J101" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 超颖电子（603175）归入“AI算力PCB+存储芯片+汽车电子板”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K101" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.9 倍，资金参与度显著放大。短中期均线保持多头排列，价格结构与趋势方向一致。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L101" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B102" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C102" s="0">
+        <v>37</v>
+      </c>
+      <c r="D102" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">001373</t>
+        </is>
+      </c>
+      <c r="E102" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">翔腾新材</t>
+        </is>
+      </c>
+      <c r="F102" s="0">
+        <v>32.44</v>
+      </c>
+      <c r="G102" s="4">
+        <v>0.1000339097999321</v>
+      </c>
+      <c r="H102" s="4">
+        <v>0.11517526054749688</v>
+      </c>
+      <c r="I102" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J102" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 翔腾新材（001373）归入“偏光片+光学膜片+MiniLED”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K102" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.9 倍，资金参与度显著放大。5日均线仍高于10日均线，但中期趋势强度一般。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L102" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B103" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C103" s="0">
+        <v>38</v>
+      </c>
+      <c r="D103" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600325</t>
+        </is>
+      </c>
+      <c r="E103" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">华发股份</t>
+        </is>
+      </c>
+      <c r="F103" s="0">
+        <v>2.73</v>
+      </c>
+      <c r="G103" s="4">
+        <v>0.10080645161290323</v>
+      </c>
+      <c r="H103" s="4">
+        <v>0.11363207665999002</v>
+      </c>
+      <c r="I103" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J103" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 华发股份（600325）归入“房地产+冰雪经济+定增”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K103" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.9 倍，资金参与度显著放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L103" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日振幅较大</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B104" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C104" s="0">
+        <v>39</v>
+      </c>
+      <c r="D104" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002860</t>
+        </is>
+      </c>
+      <c r="E104" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">星帅尔</t>
+        </is>
+      </c>
+      <c r="F104" s="0">
+        <v>18.39</v>
+      </c>
+      <c r="G104" s="4">
+        <v>0.09988038277511979</v>
+      </c>
+      <c r="H104" s="4">
+        <v>0.11309807028350415</v>
+      </c>
+      <c r="I104" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J104" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 星帅尔（002860）归入“光伏组件+家电零部件+高效电机”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K104" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.8 倍，存在明显放量。5日均线仍高于10日均线，但中期趋势强度一般。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L104" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B105" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C105" s="0">
+        <v>40</v>
+      </c>
+      <c r="D105" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603258</t>
+        </is>
+      </c>
+      <c r="E105" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">电魂网络</t>
+        </is>
+      </c>
+      <c r="F105" s="0">
+        <v>14.19</v>
+      </c>
+      <c r="G105" s="4">
+        <v>0.09999999999999985</v>
+      </c>
+      <c r="H105" s="4">
+        <v>0.11224237226615294</v>
+      </c>
+      <c r="I105" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J105" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 电魂网络（603258）归入“人工智能游戏+修仙时代+网络游戏”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K105" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.6 倍，存在明显放量。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L105" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B106" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C106" s="0">
+        <v>41</v>
+      </c>
+      <c r="D106" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002795</t>
+        </is>
+      </c>
+      <c r="E106" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">永和智控</t>
+        </is>
+      </c>
+      <c r="F106" s="0">
+        <v>8.04</v>
+      </c>
+      <c r="G106" s="4">
+        <v>0.09986320109439116</v>
+      </c>
+      <c r="H106" s="4">
+        <v>0.11179183978497693</v>
+      </c>
+      <c r="I106" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J106" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 永和智控（002795）归入“水暖阀门+医疗器械+资产出售+业绩扭亏”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K106" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 2.6 倍，资金参与度显著放大。短中期均线保持多头排列，价格结构与趋势方向一致。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L106" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B107" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C107" s="0">
+        <v>42</v>
+      </c>
+      <c r="D107" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600714</t>
+        </is>
+      </c>
+      <c r="E107" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">金瑞矿业</t>
+        </is>
+      </c>
+      <c r="F107" s="0">
+        <v>19.25</v>
+      </c>
+      <c r="G107" s="4">
+        <v>0.10000000000000009</v>
+      </c>
+      <c r="H107" s="4">
+        <v>0.10888589363275825</v>
+      </c>
+      <c r="I107" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J107" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 金瑞矿业（600714）归入“碳酸锶+锶盐扩产+玻璃基板+国家电投”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K107" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 0.6 倍，量能未出现极端放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L107" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B108" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C108" s="0">
+        <v>43</v>
+      </c>
+      <c r="D108" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600785</t>
+        </is>
+      </c>
+      <c r="E108" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">新华百货</t>
+        </is>
+      </c>
+      <c r="F108" s="0">
+        <v>11.35</v>
+      </c>
+      <c r="G108" s="4">
+        <v>0.09980620155038755</v>
+      </c>
+      <c r="H108" s="4">
+        <v>0.10654790904146405</v>
+      </c>
+      <c r="I108" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J108" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 新华百货（600785）归入“零售+智能家居+股份回购”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K108" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 0.5 倍，量能未出现极端放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L108" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B109" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C109" s="0">
+        <v>44</v>
+      </c>
+      <c r="D109" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603580</t>
+        </is>
+      </c>
+      <c r="E109" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">艾艾精工</t>
+        </is>
+      </c>
+      <c r="F109" s="0">
+        <v>71.53</v>
+      </c>
+      <c r="G109" s="4">
+        <v>0.09995386744579428</v>
+      </c>
+      <c r="H109" s="4">
+        <v>0.10652378462237674</v>
+      </c>
+      <c r="I109" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J109" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 艾艾精工（603580）归入“轻型输送带+精密金属结构件+控制权拟变更”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K109" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 0.8 倍，量能未出现极端放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L109" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B110" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C110" s="0">
+        <v>45</v>
+      </c>
+      <c r="D110" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002349</t>
+        </is>
+      </c>
+      <c r="E110" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">精华制药</t>
+        </is>
+      </c>
+      <c r="F110" s="0">
+        <v>8.71</v>
+      </c>
+      <c r="G110" s="4">
+        <v>0.09974747474747492</v>
+      </c>
+      <c r="H110" s="4">
+        <v>0.10627334237847577</v>
+      </c>
+      <c r="I110" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J110" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 精华制药（002349）归入“中药独家品种+AI制药+外用剂型”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K110" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.1 倍，量能未出现极端放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L110" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B111" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C111" s="0">
+        <v>46</v>
+      </c>
+      <c r="D111" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603395</t>
+        </is>
+      </c>
+      <c r="E111" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中盐红四方</t>
+        </is>
+      </c>
+      <c r="F111" s="0">
+        <v>28.14</v>
+      </c>
+      <c r="G111" s="4">
+        <v>0.10007818608287744</v>
+      </c>
+      <c r="H111" s="4">
+        <v>0.10535244752672822</v>
+      </c>
+      <c r="I111" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J111" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 中盐红四方（603395）归入“复合肥+新疆项目+央企”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K111" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.0 倍，量能未出现极端放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L111" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B112" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C112" s="0">
+        <v>47</v>
+      </c>
+      <c r="D112" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002622</t>
+        </is>
+      </c>
+      <c r="E112" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">皓宸医疗</t>
+        </is>
+      </c>
+      <c r="F112" s="0">
+        <v>2.72</v>
+      </c>
+      <c r="G112" s="4">
+        <v>0.10121457489878537</v>
+      </c>
+      <c r="H112" s="4">
+        <v>0.10512519825974313</v>
+      </c>
+      <c r="I112" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J112" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 皓宸医疗（002622）归入“口腔医疗+连锁服务+半年报减亏”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K112" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.9 倍，资金参与度显著放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L112" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B113" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C113" s="0">
+        <v>48</v>
+      </c>
+      <c r="D113" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">605196</t>
+        </is>
+      </c>
+      <c r="E113" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">华通线缆</t>
+        </is>
+      </c>
+      <c r="F113" s="0">
+        <v>34.62</v>
+      </c>
+      <c r="G113" s="4">
+        <v>0.100095328884652</v>
+      </c>
+      <c r="H113" s="4">
+        <v>0.10421138398395025</v>
+      </c>
+      <c r="I113" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J113" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 华通线缆（605196）归入“电线电缆+电解铝+油服产品+海外订单”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K113" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.5 倍，存在明显放量。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L113" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B114" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C114" s="0">
+        <v>49</v>
+      </c>
+      <c r="D114" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">000756</t>
+        </is>
+      </c>
+      <c r="E114" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">新华制药</t>
+        </is>
+      </c>
+      <c r="F114" s="0">
+        <v>14.67</v>
+      </c>
+      <c r="G114" s="4">
+        <v>0.09970014992503738</v>
+      </c>
+      <c r="H114" s="4">
+        <v>0.10355953792160928</v>
+      </c>
+      <c r="I114" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J114" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 新华制药（000756）归入“药品注册+阿尔茨海默病+解热镇痛”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K114" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 2.7 倍，资金参与度显著放大。5日均线仍高于10日均线，但中期趋势强度一般。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L114" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B115" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C115" s="0">
+        <v>50</v>
+      </c>
+      <c r="D115" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603289</t>
+        </is>
+      </c>
+      <c r="E115" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">泰瑞机器</t>
+        </is>
+      </c>
+      <c r="F115" s="0">
+        <v>10.51</v>
+      </c>
+      <c r="G115" s="4">
+        <v>0.10052356020942387</v>
+      </c>
+      <c r="H115" s="4">
+        <v>0.10309535830565501</v>
+      </c>
+      <c r="I115" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J115" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 泰瑞机器（603289）归入“一体化压铸+汽车注塑+海外业务”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K115" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 3.3 倍，资金参与度显著放大。短中期均线保持多头排列，价格结构与趋势方向一致。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L115" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B116" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C116" s="0">
+        <v>51</v>
+      </c>
+      <c r="D116" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603958</t>
+        </is>
+      </c>
+      <c r="E116" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">哈森股份</t>
+        </is>
+      </c>
+      <c r="F116" s="0">
+        <v>18.37</v>
+      </c>
+      <c r="G116" s="4">
+        <v>0.10000000000000009</v>
+      </c>
+      <c r="H116" s="4">
+        <v>0.10098199942322085</v>
+      </c>
+      <c r="I116" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J116" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 哈森股份（603958）归入“3D打印+苹果产业链+机器人+资产重组”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K116" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 0.9 倍，量能未出现极端放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L116" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B117" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C117" s="0">
+        <v>52</v>
+      </c>
+      <c r="D117" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600503</t>
+        </is>
+      </c>
+      <c r="E117" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">华丽家族</t>
+        </is>
+      </c>
+      <c r="F117" s="0">
+        <v>2.43</v>
+      </c>
+      <c r="G117" s="4">
+        <v>0.09954751131221728</v>
+      </c>
+      <c r="H117" s="4">
+        <v>0.09767660906243784</v>
+      </c>
+      <c r="I117" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J117" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 华丽家族（600503）归入“房地产+创新药+机器人”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K117" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 2.6 倍，资金参与度显著放大。5日均线仍高于10日均线，但中期趋势强度一般。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L117" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B118" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C118" s="0">
+        <v>53</v>
+      </c>
+      <c r="D118" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600613</t>
+        </is>
+      </c>
+      <c r="E118" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">神奇制药</t>
+        </is>
+      </c>
+      <c r="F118" s="0">
+        <v>9.25</v>
+      </c>
+      <c r="G118" s="4">
+        <v>0.0998810939357908</v>
+      </c>
+      <c r="H118" s="4">
+        <v>0.09672551632117354</v>
+      </c>
+      <c r="I118" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J118" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 神奇制药（600613）归入“抗肿瘤药+化学制药+研发推进”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K118" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 0.8 倍，量能未出现极端放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L118" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B119" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C119" s="0">
+        <v>54</v>
+      </c>
+      <c r="D119" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002900</t>
+        </is>
+      </c>
+      <c r="E119" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">哈三联</t>
+        </is>
+      </c>
+      <c r="F119" s="0">
+        <v>13.04</v>
+      </c>
+      <c r="G119" s="4">
+        <v>0.10042194092827007</v>
+      </c>
+      <c r="H119" s="4">
+        <v>0.09543416738935327</v>
+      </c>
+      <c r="I119" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J119" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 哈三联（002900）归入“创新药+化学制药+半年报减亏”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K119" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.5 倍，存在明显放量。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L119" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B120" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C120" s="0">
+        <v>55</v>
+      </c>
+      <c r="D120" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">000829</t>
+        </is>
+      </c>
+      <c r="E120" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">天音控股</t>
+        </is>
+      </c>
+      <c r="F120" s="0">
+        <v>9.77</v>
+      </c>
+      <c r="G120" s="4">
+        <v>0.10022522522522515</v>
+      </c>
+      <c r="H120" s="4">
+        <v>0.09437593703049083</v>
+      </c>
+      <c r="I120" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J120" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 天音控股（000829）归入“智能终端销售+鸿蒙生态+零售电商”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K120" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 2.8 倍，资金参与度显著放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L120" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B121" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C121" s="0">
+        <v>56</v>
+      </c>
+      <c r="D121" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">000566</t>
+        </is>
+      </c>
+      <c r="E121" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">海南海药</t>
+        </is>
+      </c>
+      <c r="F121" s="0">
+        <v>5.07</v>
+      </c>
+      <c r="G121" s="4">
+        <v>0.09978308026030369</v>
+      </c>
+      <c r="H121" s="4">
+        <v>0.09245835384523732</v>
+      </c>
+      <c r="I121" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J121" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 海南海药（000566）归入“创新药+化学制药+脑机接口+国资背景”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K121" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.7 倍，存在明显放量。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L121" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B122" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C122" s="0">
+        <v>57</v>
+      </c>
+      <c r="D122" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">000995</t>
+        </is>
+      </c>
+      <c r="E122" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">皇台酒业</t>
+        </is>
+      </c>
+      <c r="F122" s="0">
+        <v>11.92</v>
+      </c>
+      <c r="G122" s="4">
+        <v>0.09963099630996307</v>
+      </c>
+      <c r="H122" s="4">
+        <v>0.09219350106048056</v>
+      </c>
+      <c r="I122" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J122" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 皇台酒业（000995）归入“白酒+区域品牌+线上渠道”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K122" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.7 倍，存在明显放量。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L122" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B123" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C123" s="0">
+        <v>58</v>
+      </c>
+      <c r="D123" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600992</t>
+        </is>
+      </c>
+      <c r="E123" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">贵绳股份</t>
+        </is>
+      </c>
+      <c r="F123" s="0">
+        <v>10.57</v>
+      </c>
+      <c r="G123" s="4">
+        <v>0.09989594172736747</v>
+      </c>
+      <c r="H123" s="4">
+        <v>0.089757982561971</v>
+      </c>
+      <c r="I123" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J123" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 贵绳股份（600992）归入“商业航天+钢丝绳+军工+贵州国资”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K123" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 3.3 倍，资金参与度显著放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L123" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B124" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C124" s="0">
+        <v>59</v>
+      </c>
+      <c r="D124" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002907</t>
+        </is>
+      </c>
+      <c r="E124" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">华森制药</t>
+        </is>
+      </c>
+      <c r="F124" s="0">
+        <v>15.25</v>
+      </c>
+      <c r="G124" s="4">
+        <v>0.1002886002886003</v>
+      </c>
+      <c r="H124" s="4">
+        <v>0.08924696878323685</v>
+      </c>
+      <c r="I124" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J124" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 华森制药（002907）归入“创新药+青光眼+基本药物+中成药”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K124" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 1.6 倍，存在明显放量。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L124" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B125" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C125" s="0">
+        <v>60</v>
+      </c>
+      <c r="D125" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002869</t>
+        </is>
+      </c>
+      <c r="E125" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">金溢科技</t>
+        </is>
+      </c>
+      <c r="F125" s="0">
+        <v>17.04</v>
+      </c>
+      <c r="G125" s="4">
+        <v>0.1000645577792123</v>
+      </c>
+      <c r="H125" s="4">
+        <v>0.08510548454553901</v>
+      </c>
+      <c r="I125" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J125" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 金溢科技（002869）归入“车路协同+电子收费+低空智联”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K125" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 3.0 倍，资金参与度显著放大。5日均线仍高于10日均线，但中期趋势强度一般。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L125" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B126" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C126" s="0">
+        <v>61</v>
+      </c>
+      <c r="D126" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600894</t>
+        </is>
+      </c>
+      <c r="E126" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">广日股份</t>
+        </is>
+      </c>
+      <c r="F126" s="0">
+        <v>7.92</v>
+      </c>
+      <c r="G126" s="4">
+        <v>0.09999999999999985</v>
+      </c>
+      <c r="H126" s="4">
+        <v>0.08414283872293986</v>
+      </c>
+      <c r="I126" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J126" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 广日股份（600894）归入“电梯+智慧楼宇+国资背景”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K126" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 3.1 倍，资金参与度显著放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L126" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B127" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C127" s="0">
+        <v>62</v>
+      </c>
+      <c r="D127" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600281</t>
+        </is>
+      </c>
+      <c r="E127" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">华阳新材</t>
+        </is>
+      </c>
+      <c r="F127" s="0">
+        <v>4.98</v>
+      </c>
+      <c r="G127" s="4">
+        <v>0.09933774834437091</v>
+      </c>
+      <c r="H127" s="4">
+        <v>0.08157317788116751</v>
+      </c>
+      <c r="I127" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J127" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 华阳新材（600281）归入“贵金属回收+铂族金属加工+山西国资”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K127" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 0.9 倍，量能未出现极端放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L127" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">主要风险来自次日板块分歧与个股承接强弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B128" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C128" s="0">
+        <v>63</v>
+      </c>
+      <c r="D128" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002178</t>
+        </is>
+      </c>
+      <c r="E128" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">延华智能</t>
+        </is>
+      </c>
+      <c r="F128" s="0">
+        <v>5.08</v>
+      </c>
+      <c r="G128" s="4">
+        <v>0.09956709956709965</v>
+      </c>
+      <c r="H128" s="4">
+        <v>0.0797134481063416</v>
+      </c>
+      <c r="I128" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J128" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 延华智能（002178）归入“AI医疗+智慧城市+智慧康养”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K128" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 3.9 倍，资金参与度显著放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L128" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B129" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C129" s="0">
+        <v>64</v>
+      </c>
+      <c r="D129" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002755</t>
+        </is>
+      </c>
+      <c r="E129" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">奥赛康</t>
+        </is>
+      </c>
+      <c r="F129" s="0">
+        <v>12.45</v>
+      </c>
+      <c r="G129" s="4">
+        <v>0.09982332155477014</v>
+      </c>
+      <c r="H129" s="4">
+        <v>0.0760852895041779</v>
+      </c>
+      <c r="I129" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J129" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 奥赛康（002755）归入“创新药+抗感染药+肿瘤管线”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K129" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 2.8 倍，资金参与度显著放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L129" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B130" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C130" s="0">
+        <v>65</v>
+      </c>
+      <c r="D130" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002259</t>
+        </is>
+      </c>
+      <c r="E130" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">升达林业</t>
+        </is>
+      </c>
+      <c r="F130" s="0">
+        <v>4.52</v>
+      </c>
+      <c r="G130" s="4">
+        <v>0.09975669099756669</v>
+      </c>
+      <c r="H130" s="4">
+        <v>0.07587901403200374</v>
+      </c>
+      <c r="I130" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J130" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 升达林业（002259）归入“天然气+LNG加工”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K130" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 2.8 倍，资金参与度显著放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L130" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B131" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C131" s="0">
+        <v>66</v>
+      </c>
+      <c r="D131" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002022</t>
+        </is>
+      </c>
+      <c r="E131" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">科华生物</t>
+        </is>
+      </c>
+      <c r="F131" s="0">
+        <v>6.17</v>
+      </c>
+      <c r="G131" s="4">
+        <v>0.09982174688057042</v>
+      </c>
+      <c r="H131" s="4">
+        <v>0.07350526141615919</v>
+      </c>
+      <c r="I131" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J131" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 科华生物（002022）归入“体外诊断+流感检测+海外拓展”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K131" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 3.9 倍，资金参与度显著放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L131" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B132" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C132" s="0">
+        <v>67</v>
+      </c>
+      <c r="D132" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002042</t>
+        </is>
+      </c>
+      <c r="E132" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">华孚时尚</t>
+        </is>
+      </c>
+      <c r="F132" s="0">
+        <v>4.22</v>
+      </c>
+      <c r="G132" s="4">
+        <v>0.09895833333333325</v>
+      </c>
+      <c r="H132" s="4">
+        <v>0.07342317012570491</v>
+      </c>
+      <c r="I132" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J132" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 华孚时尚（002042）归入“算力租赁+色纺纱+半年报增长”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K132" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 2.4 倍，资金参与度显著放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L132" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B133" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C133" s="0">
+        <v>68</v>
+      </c>
+      <c r="D133" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600812</t>
+        </is>
+      </c>
+      <c r="E133" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">华北制药</t>
+        </is>
+      </c>
+      <c r="F133" s="0">
+        <v>5.08</v>
+      </c>
+      <c r="G133" s="4">
+        <v>0.09956709956709965</v>
+      </c>
+      <c r="H133" s="4">
+        <v>0.07219771331434721</v>
+      </c>
+      <c r="I133" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J133" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 华北制药（600812）归入“抗生素+创新药+海外市场”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K133" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 2.5 倍，资金参与度显著放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L133" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B134" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C134" s="0">
+        <v>69</v>
+      </c>
+      <c r="D134" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">000402</t>
+        </is>
+      </c>
+      <c r="E134" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">金 融 街</t>
+        </is>
+      </c>
+      <c r="F134" s="0">
+        <v>2.77</v>
+      </c>
+      <c r="G134" s="4">
+        <v>0.0992063492063493</v>
+      </c>
+      <c r="H134" s="4">
+        <v>0.07181074637154793</v>
+      </c>
+      <c r="I134" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J134" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 金 融 街（000402）归入“房地产+城市更新+北京国资”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K134" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 2.8 倍，资金参与度显著放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L134" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B135" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C135" s="0">
+        <v>70</v>
+      </c>
+      <c r="D135" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600587</t>
+        </is>
+      </c>
+      <c r="E135" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">新华医疗</t>
+        </is>
+      </c>
+      <c r="F135" s="0">
+        <v>13.4</v>
+      </c>
+      <c r="G135" s="4">
+        <v>0.10016420361247945</v>
+      </c>
+      <c r="H135" s="4">
+        <v>0.06955262861834076</v>
+      </c>
+      <c r="I135" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J135" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 新华医疗（600587）归入“康复医疗+医疗器械+脑机接口+康复机器人”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K135" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 4.9 倍，资金参与度显著放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L135" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B136" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C136" s="0">
+        <v>71</v>
+      </c>
+      <c r="D136" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603636</t>
+        </is>
+      </c>
+      <c r="E136" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">南威软件</t>
+        </is>
+      </c>
+      <c r="F136" s="0">
+        <v>7.28</v>
+      </c>
+      <c r="G136" s="4">
+        <v>0.09969788519637458</v>
+      </c>
+      <c r="H136" s="4">
+        <v>0.06324280779073169</v>
+      </c>
+      <c r="I136" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J136" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 南威软件（603636）归入“AI应用+算力租赁+政务数字化”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K136" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 4.9 倍，资金参与度显著放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L136" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B137" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C137" s="0">
+        <v>72</v>
+      </c>
+      <c r="D137" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600218</t>
+        </is>
+      </c>
+      <c r="E137" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">全柴动力</t>
+        </is>
+      </c>
+      <c r="F137" s="0">
+        <v>8.27</v>
+      </c>
+      <c r="G137" s="4">
+        <v>0.0997340425531914</v>
+      </c>
+      <c r="H137" s="4">
+        <v>0.06154928384555261</v>
+      </c>
+      <c r="I137" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">theme_only</t>
+        </is>
+      </c>
+      <c r="J137" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">题材归因标签只能说明当日市场将 全柴动力（600218）归入“柴油机+氢燃料电池+国企背景”这一交易线索，不能单独证明涨停的直接原因。需要结合公告、新闻或公司披露进一步确认。</t>
+        </is>
+      </c>
+      <c r="K137" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">收盘贴近日内最高价，说明涨停日尾盘价格维持强势。截至运行时成交量约为20日均量的 5.6 倍，资金参与度显著放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L137" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B138" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="C138" s="0">
+        <v>73</v>
+      </c>
+      <c r="D138" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600383</t>
+        </is>
+      </c>
+      <c r="E138" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">金地集团</t>
+        </is>
+      </c>
+      <c r="F138" s="0">
+        <v>2.47</v>
+      </c>
+      <c r="G138" s="4">
+        <v>0.09777777777777796</v>
+      </c>
+      <c r="H138" s="4">
+        <v>0.03521197211194885</v>
+      </c>
+      <c r="I138" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no_verified_event</t>
+        </is>
+      </c>
+      <c r="J138" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">事件证据层未找到与当日涨停直接匹配的公告或新闻；系统不把概念标签、技术形态或主观猜测当成涨停原因。</t>
+        </is>
+      </c>
+      <c r="K138" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">截至运行时成交量约为20日均量的 3.4 倍，资金参与度显著放大。短期均线未形成明显多头排列，趋势确认度相对有限。截至本次运行，市场共有 94 家涨停，其中首板 73 家、2板及以上 21 家。</t>
+        </is>
+      </c>
+      <c r="L138" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当日成交量明显放大，筹码交换较充分；当日振幅较大</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M13"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
@@ -3688,6 +7630,596 @@
       <c r="M3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">次日收盘价</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">001376</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">百通能源</t>
+        </is>
+      </c>
+      <c r="F4" s="4">
+        <v>0.4337329973097727</v>
+      </c>
+      <c r="G4" s="4">
+        <v>0.09715639810426535</v>
+      </c>
+      <c r="H4" s="4">
+        <v>0.10031595576619279</v>
+      </c>
+      <c r="I4" s="4">
+        <v>0.10031595576619279</v>
+      </c>
+      <c r="J4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="K4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">晋级二板；次日收盘相对首板收盘 +10.03%</t>
+        </is>
+      </c>
+      <c r="L4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+      <c r="M4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13.93</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603686</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">福龙马</t>
+        </is>
+      </c>
+      <c r="F5" s="4">
+        <v>0.4142972475302373</v>
+      </c>
+      <c r="G5" s="4">
+        <v>0.08920491273432463</v>
+      </c>
+      <c r="H5" s="4">
+        <v>0.08920491273432463</v>
+      </c>
+      <c r="I5" s="4">
+        <v>-0.01616031027795739</v>
+      </c>
+      <c r="J5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">否</t>
+        </is>
+      </c>
+      <c r="K5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未晋级二板；次日收盘相对首板收盘 -1.62%</t>
+        </is>
+      </c>
+      <c r="L5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+      <c r="M5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15.22</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">601579</t>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">会稽山</t>
+        </is>
+      </c>
+      <c r="F6" s="4">
+        <v>0.19249348873054756</v>
+      </c>
+      <c r="G6" s="4">
+        <v>0.020097442143726996</v>
+      </c>
+      <c r="H6" s="4">
+        <v>0.09987819732034087</v>
+      </c>
+      <c r="I6" s="4">
+        <v>0.09987819732034087</v>
+      </c>
+      <c r="J6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="K6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">晋级二板；次日收盘相对首板收盘 +9.99%</t>
+        </is>
+      </c>
+      <c r="L6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+      <c r="M6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">36.12</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">601086</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">国芳集团</t>
+        </is>
+      </c>
+      <c r="F7" s="4">
+        <v>0.17189143699227655</v>
+      </c>
+      <c r="G7" s="4">
+        <v>0.03175591531755928</v>
+      </c>
+      <c r="H7" s="4">
+        <v>0.10024906600249084</v>
+      </c>
+      <c r="I7" s="4">
+        <v>0.10024906600249084</v>
+      </c>
+      <c r="J7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="K7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">晋级二板；次日收盘相对首板收盘 +10.02%</t>
+        </is>
+      </c>
+      <c r="L7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+      <c r="M7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">17.67</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">002631</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">德尔未来</t>
+        </is>
+      </c>
+      <c r="F8" s="4">
+        <v>0.15676554518539035</v>
+      </c>
+      <c r="G8" s="4">
+        <v>0.0045351473922901064</v>
+      </c>
+      <c r="H8" s="4">
+        <v>0.08843537414965996</v>
+      </c>
+      <c r="I8" s="4">
+        <v>0.06878306878306883</v>
+      </c>
+      <c r="J8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">否</t>
+        </is>
+      </c>
+      <c r="K8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未晋级二板；次日收盘相对首板收盘 +6.88%</t>
+        </is>
+      </c>
+      <c r="L8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+      <c r="M8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14.14</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603353</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">和顺石油</t>
+        </is>
+      </c>
+      <c r="F9" s="4">
+        <v>0.1561549742231579</v>
+      </c>
+      <c r="G9" s="4">
+        <v>0.015036045314109181</v>
+      </c>
+      <c r="H9" s="4">
+        <v>0.06405767250257455</v>
+      </c>
+      <c r="I9" s="4">
+        <v>-0.04449021627188454</v>
+      </c>
+      <c r="J9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">否</t>
+        </is>
+      </c>
+      <c r="K9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未晋级二板；次日收盘相对首板收盘 -4.45%</t>
+        </is>
+      </c>
+      <c r="L9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+      <c r="M9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">46.39</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">001212</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">中旗新材</t>
+        </is>
+      </c>
+      <c r="F10" s="4">
+        <v>0.1560505754187151</v>
+      </c>
+      <c r="G10" s="4">
+        <v>-0.005265929436545469</v>
+      </c>
+      <c r="H10" s="4">
+        <v>0.018957345971564177</v>
+      </c>
+      <c r="I10" s="4">
+        <v>0.00868878357030023</v>
+      </c>
+      <c r="J10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">否</t>
+        </is>
+      </c>
+      <c r="K10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未晋级二板；次日收盘相对首板收盘 +0.87%</t>
+        </is>
+      </c>
+      <c r="L10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+      <c r="M10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">38.31</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603138</t>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">海量数据</t>
+        </is>
+      </c>
+      <c r="F11" s="4">
+        <v>0.15416750520049954</v>
+      </c>
+      <c r="G11" s="4">
+        <v>0.026974951830443183</v>
+      </c>
+      <c r="H11" s="4">
+        <v>0.04688503532434174</v>
+      </c>
+      <c r="I11" s="4">
+        <v>0.010918432883750828</v>
+      </c>
+      <c r="J11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">否</t>
+        </is>
+      </c>
+      <c r="K11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未晋级二板；次日收盘相对首板收盘 +1.09%</t>
+        </is>
+      </c>
+      <c r="L11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+      <c r="M11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15.74</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600343</t>
+        </is>
+      </c>
+      <c r="E12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">航天动力</t>
+        </is>
+      </c>
+      <c r="F12" s="4">
+        <v>0.15170675706937384</v>
+      </c>
+      <c r="G12" s="4">
+        <v>-0.014305491462851982</v>
+      </c>
+      <c r="H12" s="4">
+        <v>-0.006460544531610601</v>
+      </c>
+      <c r="I12" s="4">
+        <v>-0.029072450392247484</v>
+      </c>
+      <c r="J12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">否</t>
+        </is>
+      </c>
+      <c r="K12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未晋级二板；次日收盘相对首板收盘 -2.91%</t>
+        </is>
+      </c>
+      <c r="L12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+      <c r="M12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">21.04</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603316</t>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">诚邦股份</t>
+        </is>
+      </c>
+      <c r="F13" s="4">
+        <v>0.14909280780204942</v>
+      </c>
+      <c r="G13" s="4">
+        <v>0.046135410425404366</v>
+      </c>
+      <c r="H13" s="4">
+        <v>0.10005991611743537</v>
+      </c>
+      <c r="I13" s="4">
+        <v>0.10005991611743537</v>
+      </c>
+      <c r="J13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是</t>
+        </is>
+      </c>
+      <c r="K13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">晋级二板；次日收盘相对首板收盘 +10.01%</t>
+        </is>
+      </c>
+      <c r="L13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+      <c r="M13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18.36</t>
         </is>
       </c>
     </row>
@@ -3779,21 +8311,29 @@
         </is>
       </c>
       <c r="B3" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3" s="0">
-        <v>0</v>
-      </c>
-      <c r="E3" s="0"/>
-      <c r="F3" s="0"/>
-      <c r="G3" s="0"/>
+        <v>1</v>
+      </c>
+      <c r="E3" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="F3" s="4">
+        <v>0.20967741935483872</v>
+      </c>
+      <c r="G3" s="0">
+        <v>4.769230769230769</v>
+      </c>
       <c r="H3" s="0">
-        <v>0</v>
-      </c>
-      <c r="I3" s="0"/>
+        <v>1</v>
+      </c>
+      <c r="I3" s="4">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
@@ -3802,21 +8342,29 @@
         </is>
       </c>
       <c r="B4" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4" s="0">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D4" s="0">
-        <v>0</v>
-      </c>
-      <c r="E4" s="0"/>
-      <c r="F4" s="0"/>
-      <c r="G4" s="0"/>
+        <v>2</v>
+      </c>
+      <c r="E4" s="4">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="F4" s="4">
+        <v>0.20967741935483872</v>
+      </c>
+      <c r="G4" s="0">
+        <v>3.1794871794871793</v>
+      </c>
       <c r="H4" s="0">
-        <v>0</v>
-      </c>
-      <c r="I4" s="0"/>
+        <v>1</v>
+      </c>
+      <c r="I4" s="4">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
@@ -3825,21 +8373,29 @@
         </is>
       </c>
       <c r="B5" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C5" s="0">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D5" s="0">
-        <v>0</v>
-      </c>
-      <c r="E5" s="0"/>
-      <c r="F5" s="0"/>
-      <c r="G5" s="0"/>
+        <v>3</v>
+      </c>
+      <c r="E5" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="F5" s="4">
+        <v>0.20967741935483872</v>
+      </c>
+      <c r="G5" s="0">
+        <v>2.3846153846153846</v>
+      </c>
       <c r="H5" s="0">
-        <v>0</v>
-      </c>
-      <c r="I5" s="0"/>
+        <v>1</v>
+      </c>
+      <c r="I5" s="4">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
@@ -3848,21 +8404,29 @@
         </is>
       </c>
       <c r="B6" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6" s="0">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D6" s="0">
-        <v>0</v>
-      </c>
-      <c r="E6" s="0"/>
-      <c r="F6" s="0"/>
-      <c r="G6" s="0"/>
+        <v>4</v>
+      </c>
+      <c r="E6" s="4">
+        <v>0.4</v>
+      </c>
+      <c r="F6" s="4">
+        <v>0.20967741935483872</v>
+      </c>
+      <c r="G6" s="0">
+        <v>1.9076923076923078</v>
+      </c>
       <c r="H6" s="0">
-        <v>0</v>
-      </c>
-      <c r="I6" s="0"/>
+        <v>1</v>
+      </c>
+      <c r="I6" s="4">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">

</xml_diff>